<commit_message>
7/04 - first edits
</commit_message>
<xml_diff>
--- a/data/monthly_cru_data.xlsx
+++ b/data/monthly_cru_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mollyotoole/SCIE3121_Molly_OToole/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7FAD2A3F-31A0-624C-857D-06D63537EFF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFCCC60D-B75A-EF4C-9C12-0658BD5ADD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="720" yWindow="500" windowWidth="28080" windowHeight="16420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="500" windowWidth="26880" windowHeight="16420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tas" sheetId="1" r:id="rId1"/>

</xml_diff>